<commit_message>
New tests, and fixes and updates to existing tests
</commit_message>
<xml_diff>
--- a/cms/metrics_documentation/data_migration/source_data/metrics_definitions_migration_edit.xlsx
+++ b/cms/metrics_documentation/data_migration/source_data/metrics_definitions_migration_edit.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ian.rufus/hsa/data-dashboard-api/cms/metrics_documentation/data_migration/source_data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD046834-913F-6340-95A7-155E20FE7543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="2440" yWindow="3780" windowWidth="58940" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="289">
   <si>
     <t>Title</t>
   </si>
@@ -205,6 +214,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -214,6 +224,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -223,6 +234,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -232,6 +244,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -241,6 +254,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -250,6 +264,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -259,6 +274,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -268,6 +284,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -277,6 +294,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">There is a lag of at least 11 days in the reporting of data </t>
     </r>
@@ -285,6 +303,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>and the 14 days prior to the latest date available in the dataset is considered to be incomplete</t>
     </r>
@@ -293,6 +312,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> due to the time taken for deaths to be registered.
 </t>
@@ -302,6 +322,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -311,6 +332,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The count of reported new deaths in the last 7 days is the total of the daily deaths registered in the 7 days up to and including the most recent date with "complete" data.  </t>
     </r>
@@ -337,6 +359,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -346,6 +369,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -355,6 +379,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -364,6 +389,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -373,6 +399,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -382,6 +409,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -391,6 +419,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -400,6 +429,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -409,6 +439,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">There is a lag of at least 11 days in the reporting of data </t>
     </r>
@@ -417,6 +448,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>and the 14 days prior to the latest date available in the dataset is considered to be incomplete</t>
     </r>
@@ -425,6 +457,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> due to the time taken for deaths to be registered.
 </t>
@@ -434,6 +467,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -443,6 +477,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The change in new deaths in the last 7 days is the difference between the total of the daily deaths registered in the 7 days up to and including the most recent date with "complete" data and the total of the daily deaths registered in the previous 7 days. </t>
     </r>
@@ -466,6 +501,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -475,6 +511,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -484,6 +521,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -493,6 +531,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -502,6 +541,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -511,6 +551,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -520,6 +561,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -529,6 +571,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -538,6 +581,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>There is a lag of at least 11 days in the reporting of data</t>
     </r>
@@ -546,6 +590,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> and the 14 days prior to the latest date available in the dataset is considered to be incomplete</t>
     </r>
@@ -554,6 +599,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> due to the time taken for deaths to be registered.
 </t>
@@ -563,6 +609,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -572,6 +619,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">The percentage change in new deaths in the last 7 days is calculated as the difference between the total of the daily deaths registered in the 7 days up to and including the most recent date with "complete" data and the total of the daily deaths registered in the previous 7 days, divided by the total of the daily deaths registered in the previous 7 days.  
 </t>
@@ -600,6 +648,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -609,6 +658,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -618,6 +668,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -627,6 +678,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -636,6 +688,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -645,6 +698,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -654,6 +708,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -663,6 +718,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -672,6 +728,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">There is a lag of at least 11 days in the reporting of data </t>
     </r>
@@ -680,6 +737,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">and the 14 days prior to the latest date available in the dataset is considered to be incomplete </t>
     </r>
@@ -688,6 +746,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>due to the time taken for deaths to be registered.</t>
     </r>
@@ -711,6 +770,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -720,6 +780,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -729,6 +790,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -738,6 +800,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -747,6 +810,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -756,6 +820,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -765,6 +830,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -774,6 +840,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -783,6 +850,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">There is a lag of at least 11 days in the reporting of data </t>
     </r>
@@ -791,6 +859,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>and the 14 days prior to the latest date available in the dataset is considered to be incomplete</t>
     </r>
@@ -799,6 +868,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> due to the time taken for deaths to be registered.
 </t>
@@ -808,6 +878,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -817,6 +888,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>The value shown on a given date is the total of the deaths registered in the 7 days up to and including that date divided by 7.</t>
     </r>
@@ -840,6 +912,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths where COVID-19 is mentioned as one of the causes on the death certificate are reported by the Office for National Statistics.
 </t>
@@ -849,6 +922,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -858,6 +932,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> The deceased may or may not have had a confirmed positive test for COVID-19. People who had COVID-19 but did not have it mentioned on their death certificate as a cause of death are excluded.
 </t>
@@ -867,6 +942,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -876,6 +952,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Deaths are allocated to the deceased's usual area of residence.
 </t>
@@ -885,6 +962,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -894,6 +972,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Bank holidays can affect the number of deaths registered in a given week.
 </t>
@@ -903,6 +982,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -912,6 +992,7 @@
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>There is a lag of at least 11 days in the reporting of data</t>
     </r>
@@ -920,6 +1001,7 @@
         <sz val="11"/>
         <color indexed="13"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> and the 14 days prior to the latest date available in the dataset is considered to be incomplete due to the time taken for deaths to be registered.</t>
     </r>
@@ -1679,55 +1761,56 @@
 Updates from SARI Watch are published in the UKHSA National Influenza and COVID-19 Surveillance Report on a Friday (weekly during influenza season and fortnightly in the summer months), and contains data up to the previous Sunday. 
 Weekly positivity is calculated as the count of number of PCR tests taken in the last 7 days up to and including the date shown which had a positive result, divided by the total number of positive or negative PCR tests taken in the last 7 days up to and including the date shown.</t>
   </si>
+  <si>
+    <t>Id</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="13"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="15"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="15"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1780,7 +1863,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1868,99 +1951,111 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+  <cellXfs count="32">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1970,32 +2065,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffc5deb5"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="fffff2cc"/>
-      <rgbColor rgb="ffbdd7ee"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ffdac2ec"/>
-      <rgbColor rgb="ff0b0c0c"/>
-      <rgbColor rgb="fffce4d6"/>
-      <rgbColor rgb="ffffafcf"/>
-      <rgbColor rgb="fffbe4d5"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFC5DEB5"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFBDD7EE"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFDAC2EC"/>
+      <rgbColor rgb="FF0B0C0C"/>
+      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFFFAFCF"/>
+      <rgbColor rgb="FFFBE4D5"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office Theme">
       <a:dk1>
@@ -2197,7 +2345,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -2216,7 +2364,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2246,7 +2394,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2272,7 +2420,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2298,7 +2446,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2324,7 +2472,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2350,7 +2498,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2376,7 +2524,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2402,7 +2550,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2428,7 +2576,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2454,7 +2602,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2467,9 +2615,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -2486,7 +2640,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -2505,7 +2659,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2531,7 +2685,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2557,7 +2711,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2583,7 +2737,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2609,7 +2763,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2635,7 +2789,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2661,7 +2815,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2687,7 +2841,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2713,7 +2867,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2739,7 +2893,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2752,9 +2906,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -2768,7 +2928,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -2787,7 +2947,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2817,7 +2977,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2843,7 +3003,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2869,7 +3029,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2895,7 +3055,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2921,7 +3081,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2947,7 +3107,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2973,7 +3133,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2999,7 +3159,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -3025,7 +3185,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -3038,1270 +3198,1446 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G56"/>
-  <sheetFormatPr defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H56"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.1719" style="1" customWidth="1"/>
-    <col min="3" max="3" width="62.6719" style="1" customWidth="1"/>
-    <col min="4" max="4" width="108.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="106.172" style="1" customWidth="1"/>
-    <col min="6" max="6" width="91.6719" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="62.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="73.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="91.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="47" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.67188" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="3">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="4">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="4">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="4">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="3">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="3">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" ht="296" customHeight="1">
-      <c r="A2" t="s" s="5">
+      <c r="H1" s="29" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="296" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s" s="5">
+      <c r="B2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s" s="5">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s" s="5">
+      <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s" s="5">
+      <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s" s="6">
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s" s="6">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" ht="255.5" customHeight="1">
-      <c r="A3" t="s" s="5">
+      <c r="H2" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="255.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s" s="5">
+      <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s" s="5">
+      <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s" s="5">
+      <c r="D3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s" s="5">
+      <c r="E3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s" s="6">
+      <c r="F3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s" s="6">
+      <c r="G3" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" ht="322.25" customHeight="1">
-      <c r="A4" t="s" s="5">
+      <c r="H3" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="322.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s" s="5">
+      <c r="B4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s" s="5">
+      <c r="C4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s" s="5">
+      <c r="D4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E4" t="s" s="5">
+      <c r="E4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F4" t="s" s="6">
+      <c r="F4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G4" t="s" s="6">
+      <c r="G4" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" ht="257.75" customHeight="1">
-      <c r="A5" t="s" s="5">
+      <c r="H4" s="1">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="257.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s" s="5">
+      <c r="B5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s" s="5">
+      <c r="C5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s" s="5">
+      <c r="D5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E5" t="s" s="5">
+      <c r="E5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F5" t="s" s="6">
+      <c r="F5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G5" t="s" s="6">
+      <c r="G5" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" ht="304" customHeight="1">
-      <c r="A6" t="s" s="5">
+      <c r="H5" s="30">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="304" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s" s="5">
+      <c r="B6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C6" t="s" s="5">
+      <c r="C6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D6" t="s" s="5">
+      <c r="D6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="s" s="5">
+      <c r="E6" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F6" t="s" s="6">
+      <c r="F6" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s" s="6">
+      <c r="G6" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" ht="304" customHeight="1">
-      <c r="A7" t="s" s="5">
+      <c r="H6" s="30">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="304" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B7" t="s" s="5">
+      <c r="B7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s" s="5">
+      <c r="C7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D7" t="s" s="7">
+      <c r="D7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E7" t="s" s="8">
+      <c r="E7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F7" t="s" s="6">
+      <c r="F7" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G7" t="s" s="6">
+      <c r="G7" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" ht="237.5" customHeight="1">
-      <c r="A8" t="s" s="9">
+      <c r="H7" s="30">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="237.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B8" t="s" s="9">
+      <c r="B8" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C8" t="s" s="9">
+      <c r="C8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s" s="9">
+      <c r="D8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s" s="9">
+      <c r="E8" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F8" t="s" s="10">
+      <c r="F8" s="10" t="s">
         <v>47</v>
       </c>
       <c r="G8" s="11"/>
-    </row>
-    <row r="9" ht="254.75" customHeight="1">
-      <c r="A9" t="s" s="9">
+      <c r="H8" s="30">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="254.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B9" t="s" s="9">
+      <c r="B9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" t="s" s="9">
+      <c r="C9" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D9" t="s" s="9">
+      <c r="D9" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E9" t="s" s="9">
+      <c r="E9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F9" t="s" s="10">
+      <c r="F9" s="10" t="s">
         <v>53</v>
       </c>
       <c r="G9" s="12"/>
-    </row>
-    <row r="10" ht="274.25" customHeight="1">
-      <c r="A10" t="s" s="9">
+      <c r="H9" s="30">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="274.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B10" t="s" s="9">
+      <c r="B10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C10" t="s" s="9">
+      <c r="C10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D10" t="s" s="9">
+      <c r="D10" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E10" t="s" s="9">
+      <c r="E10" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F10" t="s" s="10">
+      <c r="F10" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G10" t="s" s="10">
+      <c r="G10" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="11" ht="202.75" customHeight="1">
-      <c r="A11" t="s" s="9">
+      <c r="H10" s="30">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="202.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B11" t="s" s="9">
+      <c r="B11" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C11" t="s" s="9">
+      <c r="C11" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D11" t="s" s="9">
+      <c r="D11" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="E11" t="s" s="9">
+      <c r="E11" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F11" t="s" s="10">
+      <c r="F11" s="10" t="s">
         <v>64</v>
       </c>
       <c r="G11" s="12"/>
-    </row>
-    <row r="12" ht="244.75" customHeight="1">
-      <c r="A12" t="s" s="9">
+      <c r="H11" s="30">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="244.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B12" t="s" s="9">
+      <c r="B12" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C12" t="s" s="9">
+      <c r="C12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D12" t="s" s="9">
+      <c r="D12" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E12" t="s" s="9">
+      <c r="E12" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F12" t="s" s="10">
+      <c r="F12" s="10" t="s">
         <v>69</v>
       </c>
       <c r="G12" s="12"/>
-    </row>
-    <row r="13" ht="244.75" customHeight="1">
-      <c r="A13" t="s" s="9">
+      <c r="H12" s="30">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="244.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B13" t="s" s="9">
+      <c r="B13" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C13" t="s" s="9">
+      <c r="C13" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D13" t="s" s="9">
+      <c r="D13" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="E13" t="s" s="9">
+      <c r="E13" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F13" t="s" s="10">
+      <c r="F13" s="10" t="s">
         <v>74</v>
       </c>
       <c r="G13" s="12"/>
-    </row>
-    <row r="14" ht="138.5" customHeight="1">
-      <c r="A14" t="s" s="13">
+      <c r="H13" s="30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="138.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B14" t="s" s="13">
+      <c r="B14" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C14" t="s" s="13">
+      <c r="C14" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D14" t="s" s="13">
+      <c r="D14" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E14" t="s" s="13">
+      <c r="E14" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="F14" t="s" s="14">
+      <c r="F14" s="14" t="s">
         <v>79</v>
       </c>
       <c r="G14" s="15"/>
-    </row>
-    <row r="15" ht="201" customHeight="1">
-      <c r="A15" t="s" s="13">
+      <c r="H14" s="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="201" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B15" t="s" s="13">
+      <c r="B15" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C15" t="s" s="13">
+      <c r="C15" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D15" t="s" s="13">
+      <c r="D15" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E15" t="s" s="13">
+      <c r="E15" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F15" t="s" s="14">
+      <c r="F15" s="14" t="s">
         <v>84</v>
       </c>
       <c r="G15" s="15"/>
-    </row>
-    <row r="16" ht="208.75" customHeight="1">
-      <c r="A16" t="s" s="13">
+      <c r="H15" s="1">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="208.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B16" t="s" s="13">
+      <c r="B16" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="C16" t="s" s="13">
+      <c r="C16" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D16" t="s" s="13">
+      <c r="D16" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E16" t="s" s="13">
+      <c r="E16" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="F16" t="s" s="14">
+      <c r="F16" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="G16" t="s" s="14">
+      <c r="G16" s="14" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" ht="176" customHeight="1">
-      <c r="A17" t="s" s="13">
+      <c r="H16" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B17" t="s" s="13">
+      <c r="B17" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="C17" t="s" s="13">
+      <c r="C17" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D17" t="s" s="13">
+      <c r="D17" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="E17" t="s" s="13">
+      <c r="E17" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="F17" t="s" s="14">
+      <c r="F17" s="14" t="s">
         <v>92</v>
       </c>
       <c r="G17" s="16"/>
-    </row>
-    <row r="18" ht="192" customHeight="1">
-      <c r="A18" t="s" s="13">
+      <c r="H17" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B18" t="s" s="13">
+      <c r="B18" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="C18" t="s" s="13">
+      <c r="C18" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D18" t="s" s="13">
+      <c r="D18" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="E18" t="s" s="13">
+      <c r="E18" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="F18" t="s" s="14">
+      <c r="F18" s="14" t="s">
         <v>96</v>
       </c>
       <c r="G18" s="16"/>
-    </row>
-    <row r="19" ht="192" customHeight="1">
-      <c r="A19" t="s" s="13">
+      <c r="H18" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B19" t="s" s="13">
+      <c r="B19" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C19" t="s" s="13">
+      <c r="C19" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D19" t="s" s="13">
+      <c r="D19" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="E19" t="s" s="13">
+      <c r="E19" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="F19" t="s" s="14">
+      <c r="F19" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="G19" t="s" s="17">
+      <c r="G19" s="17" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="20" ht="156.5" customHeight="1">
-      <c r="A20" t="s" s="13">
+      <c r="H19" s="1">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="156.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="B20" t="s" s="13">
+      <c r="B20" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C20" t="s" s="13">
+      <c r="C20" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D20" t="s" s="13">
+      <c r="D20" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="E20" t="s" s="13">
+      <c r="E20" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="F20" t="s" s="14">
+      <c r="F20" s="14" t="s">
         <v>104</v>
       </c>
       <c r="G20" s="18"/>
-    </row>
-    <row r="21" ht="176" customHeight="1">
-      <c r="A21" t="s" s="13">
+      <c r="H20" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B21" t="s" s="13">
+      <c r="B21" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C21" t="s" s="13">
+      <c r="C21" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D21" t="s" s="13">
+      <c r="D21" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="E21" t="s" s="13">
+      <c r="E21" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="F21" t="s" s="14">
+      <c r="F21" s="14" t="s">
         <v>108</v>
       </c>
       <c r="G21" s="15"/>
-    </row>
-    <row r="22" ht="96" customHeight="1">
-      <c r="A22" t="s" s="13">
+      <c r="H21" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B22" t="s" s="13">
+      <c r="B22" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="C22" t="s" s="13">
+      <c r="C22" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D22" t="s" s="13">
+      <c r="D22" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E22" t="s" s="13">
+      <c r="E22" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="F22" t="s" s="14">
+      <c r="F22" s="14" t="s">
         <v>112</v>
       </c>
       <c r="G22" s="15"/>
-    </row>
-    <row r="23" ht="128" customHeight="1">
-      <c r="A23" t="s" s="19">
+      <c r="H22" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="128" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="B23" t="s" s="19">
+      <c r="B23" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C23" t="s" s="19">
+      <c r="C23" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D23" t="s" s="19">
+      <c r="D23" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="E23" t="s" s="19">
+      <c r="E23" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="F23" t="s" s="20">
+      <c r="F23" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="G23" t="s" s="20">
+      <c r="G23" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="24" ht="128" customHeight="1">
-      <c r="A24" t="s" s="19">
+      <c r="H23" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="128" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="B24" t="s" s="19">
+      <c r="B24" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="C24" t="s" s="19">
+      <c r="C24" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D24" t="s" s="19">
+      <c r="D24" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="E24" t="s" s="21">
+      <c r="E24" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="F24" t="s" s="20">
+      <c r="F24" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="G24" t="s" s="20">
+      <c r="G24" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="25" ht="160" customHeight="1">
-      <c r="A25" t="s" s="19">
+      <c r="H24" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="B25" t="s" s="19">
+      <c r="B25" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="C25" t="s" s="19">
+      <c r="C25" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D25" t="s" s="22">
+      <c r="D25" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="E25" t="s" s="23">
+      <c r="E25" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="F25" t="s" s="20">
+      <c r="F25" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="G25" t="s" s="20">
+      <c r="G25" s="20" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="26" ht="160" customHeight="1">
-      <c r="A26" t="s" s="19">
+      <c r="H25" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="B26" t="s" s="19">
+      <c r="B26" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C26" t="s" s="19">
+      <c r="C26" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D26" t="s" s="19">
+      <c r="D26" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="E26" t="s" s="19">
+      <c r="E26" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="F26" t="s" s="20">
+      <c r="F26" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="G26" t="s" s="20">
+      <c r="G26" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="27" ht="112" customHeight="1">
-      <c r="A27" t="s" s="19">
+      <c r="H26" s="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="B27" t="s" s="19">
+      <c r="B27" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="C27" t="s" s="19">
+      <c r="C27" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D27" t="s" s="19">
+      <c r="D27" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="E27" t="s" s="19">
+      <c r="E27" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="F27" t="s" s="20">
+      <c r="F27" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="G27" t="s" s="20">
+      <c r="G27" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="28" ht="144" customHeight="1">
-      <c r="A28" t="s" s="19">
+      <c r="H27" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="B28" t="s" s="19">
+      <c r="B28" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="C28" t="s" s="19">
+      <c r="C28" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D28" t="s" s="19">
+      <c r="D28" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E28" t="s" s="19">
+      <c r="E28" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="F28" t="s" s="20">
+      <c r="F28" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="G28" t="s" s="20">
+      <c r="G28" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="29" ht="176" customHeight="1">
-      <c r="A29" t="s" s="24">
+      <c r="H28" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="B29" t="s" s="24">
+      <c r="B29" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="C29" t="s" s="24">
+      <c r="C29" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D29" t="s" s="24">
+      <c r="D29" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="E29" t="s" s="24">
+      <c r="E29" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="F29" t="s" s="25">
+      <c r="F29" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="G29" t="s" s="25">
+      <c r="G29" s="25" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="30" ht="192" customHeight="1">
-      <c r="A30" t="s" s="24">
+      <c r="H29" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="24" t="s">
         <v>152</v>
       </c>
-      <c r="B30" t="s" s="24">
+      <c r="B30" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="C30" t="s" s="24">
+      <c r="C30" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D30" t="s" s="24">
+      <c r="D30" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="E30" t="s" s="24">
+      <c r="E30" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="F30" t="s" s="25">
+      <c r="F30" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="G30" t="s" s="25">
+      <c r="G30" s="25" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="31" ht="176" customHeight="1">
-      <c r="A31" t="s" s="24">
+      <c r="H30" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="B31" t="s" s="24">
+      <c r="B31" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="C31" t="s" s="24">
+      <c r="C31" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D31" t="s" s="24">
+      <c r="D31" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="E31" t="s" s="24">
+      <c r="E31" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="F31" t="s" s="25">
+      <c r="F31" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="G31" t="s" s="25">
+      <c r="G31" s="25" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="32" ht="192" customHeight="1">
-      <c r="A32" t="s" s="24">
+      <c r="H31" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="B32" t="s" s="24">
+      <c r="B32" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="C32" t="s" s="24">
+      <c r="C32" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D32" t="s" s="24">
+      <c r="D32" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="E32" t="s" s="24">
+      <c r="E32" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="F32" t="s" s="25">
+      <c r="F32" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="G32" t="s" s="25">
+      <c r="G32" s="25" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="33" ht="176" customHeight="1">
-      <c r="A33" t="s" s="24">
+      <c r="H32" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="B33" t="s" s="24">
+      <c r="B33" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="C33" t="s" s="24">
+      <c r="C33" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D33" t="s" s="24">
+      <c r="D33" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="E33" t="s" s="24">
+      <c r="E33" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="F33" t="s" s="25">
+      <c r="F33" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="G33" t="s" s="25">
+      <c r="G33" s="25" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="34" ht="192" customHeight="1">
-      <c r="A34" t="s" s="24">
+      <c r="H33" s="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B34" t="s" s="24">
+      <c r="B34" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="C34" t="s" s="24">
+      <c r="C34" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D34" t="s" s="24">
+      <c r="D34" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="E34" t="s" s="24">
+      <c r="E34" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="F34" t="s" s="25">
+      <c r="F34" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="G34" t="s" s="25">
+      <c r="G34" s="25" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="35" ht="176" customHeight="1">
-      <c r="A35" t="s" s="24">
+      <c r="H34" s="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="B35" t="s" s="24">
+      <c r="B35" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="C35" t="s" s="24">
+      <c r="C35" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D35" t="s" s="24">
+      <c r="D35" s="24" t="s">
         <v>177</v>
       </c>
-      <c r="E35" t="s" s="24">
+      <c r="E35" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="F35" t="s" s="25">
+      <c r="F35" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="G35" t="s" s="25">
+      <c r="G35" s="25" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="36" ht="192" customHeight="1">
-      <c r="A36" t="s" s="24">
+      <c r="H35" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="B36" t="s" s="24">
+      <c r="B36" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="C36" t="s" s="24">
+      <c r="C36" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D36" t="s" s="24">
+      <c r="D36" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="E36" t="s" s="24">
+      <c r="E36" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="F36" t="s" s="25">
+      <c r="F36" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="G36" t="s" s="25">
+      <c r="G36" s="25" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="37" ht="176" customHeight="1">
-      <c r="A37" t="s" s="24">
+      <c r="H36" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="176" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B37" t="s" s="24">
+      <c r="B37" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="C37" t="s" s="24">
+      <c r="C37" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D37" t="s" s="24">
+      <c r="D37" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="E37" t="s" s="24">
+      <c r="E37" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="F37" t="s" s="25">
+      <c r="F37" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="G37" t="s" s="25">
+      <c r="G37" s="25" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="38" ht="192" customHeight="1">
-      <c r="A38" t="s" s="24">
+      <c r="H37" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="192" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="B38" t="s" s="24">
+      <c r="B38" s="24" t="s">
         <v>192</v>
       </c>
-      <c r="C38" t="s" s="24">
+      <c r="C38" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="D38" t="s" s="24">
+      <c r="D38" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="E38" t="s" s="24">
+      <c r="E38" s="24" t="s">
         <v>194</v>
       </c>
-      <c r="F38" t="s" s="25">
+      <c r="F38" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="G38" t="s" s="25">
+      <c r="G38" s="25" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="39" ht="272" customHeight="1">
-      <c r="A39" t="s" s="13">
+      <c r="H38" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="272" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="B39" t="s" s="13">
+      <c r="B39" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="C39" t="s" s="13">
+      <c r="C39" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D39" t="s" s="13">
+      <c r="D39" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="E39" t="s" s="13">
+      <c r="E39" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="F39" t="s" s="14">
+      <c r="F39" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="G39" t="s" s="14">
+      <c r="G39" s="14" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="40" ht="272" customHeight="1">
-      <c r="A40" t="s" s="13">
+      <c r="H39" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="272" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="B40" t="s" s="13">
+      <c r="B40" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="C40" t="s" s="13">
+      <c r="C40" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D40" t="s" s="13">
+      <c r="D40" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="E40" t="s" s="13">
+      <c r="E40" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="F40" t="s" s="14">
+      <c r="F40" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="G40" t="s" s="14">
+      <c r="G40" s="14" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="41" ht="272" customHeight="1">
-      <c r="A41" t="s" s="13">
+      <c r="H40" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="272" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="B41" t="s" s="13">
+      <c r="B41" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="C41" t="s" s="13">
+      <c r="C41" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D41" t="s" s="13">
+      <c r="D41" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="E41" t="s" s="13">
+      <c r="E41" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="F41" t="s" s="14">
+      <c r="F41" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="G41" t="s" s="14">
+      <c r="G41" s="14" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="42" ht="272" customHeight="1">
-      <c r="A42" t="s" s="13">
+      <c r="H41" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="272" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="B42" t="s" s="13">
+      <c r="B42" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="C42" t="s" s="13">
+      <c r="C42" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D42" t="s" s="13">
+      <c r="D42" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E42" t="s" s="13">
+      <c r="E42" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="F42" t="s" s="14">
+      <c r="F42" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="G42" t="s" s="14">
+      <c r="G42" s="14" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="43" ht="160" customHeight="1">
-      <c r="A43" t="s" s="19">
+      <c r="H42" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="B43" t="s" s="19">
+      <c r="B43" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="C43" t="s" s="19">
+      <c r="C43" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D43" t="s" s="19">
+      <c r="D43" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="E43" t="s" s="19">
+      <c r="E43" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="F43" t="s" s="20">
+      <c r="F43" s="20" t="s">
         <v>219</v>
       </c>
       <c r="G43" s="26"/>
-    </row>
-    <row r="44" ht="160" customHeight="1">
-      <c r="A44" t="s" s="19">
+      <c r="H43" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="B44" t="s" s="19">
+      <c r="B44" s="19" t="s">
         <v>221</v>
       </c>
-      <c r="C44" t="s" s="19">
+      <c r="C44" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D44" t="s" s="19">
+      <c r="D44" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="E44" t="s" s="19">
+      <c r="E44" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="F44" t="s" s="20">
+      <c r="F44" s="20" t="s">
         <v>224</v>
       </c>
       <c r="G44" s="26"/>
-    </row>
-    <row r="45" ht="112" customHeight="1">
-      <c r="A45" t="s" s="13">
+      <c r="H44" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="B45" t="s" s="13">
+      <c r="B45" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="C45" t="s" s="13">
+      <c r="C45" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D45" t="s" s="13">
+      <c r="D45" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="E45" t="s" s="13">
+      <c r="E45" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="F45" t="s" s="14">
+      <c r="F45" s="14" t="s">
         <v>228</v>
       </c>
       <c r="G45" s="15"/>
-    </row>
-    <row r="46" ht="128" customHeight="1">
-      <c r="A46" t="s" s="13">
+      <c r="H45" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="128" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="B46" t="s" s="13">
+      <c r="B46" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="C46" t="s" s="13">
+      <c r="C46" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D46" t="s" s="13">
+      <c r="D46" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="E46" t="s" s="13">
+      <c r="E46" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="F46" t="s" s="14">
+      <c r="F46" s="14" t="s">
         <v>232</v>
       </c>
       <c r="G46" s="15"/>
-    </row>
-    <row r="47" ht="160" customHeight="1">
-      <c r="A47" t="s" s="27">
+      <c r="H46" s="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="27" t="s">
         <v>233</v>
       </c>
-      <c r="B47" t="s" s="27">
+      <c r="B47" s="27" t="s">
         <v>234</v>
       </c>
-      <c r="C47" t="s" s="27">
+      <c r="C47" s="27" t="s">
         <v>235</v>
       </c>
-      <c r="D47" t="s" s="19">
+      <c r="D47" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="E47" t="s" s="19">
+      <c r="E47" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="F47" t="s" s="20">
+      <c r="F47" s="20" t="s">
         <v>238</v>
       </c>
       <c r="G47" s="28"/>
-    </row>
-    <row r="48" ht="160" customHeight="1">
-      <c r="A48" t="s" s="27">
+      <c r="H47" s="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="B48" t="s" s="27">
+      <c r="B48" s="27" t="s">
         <v>240</v>
       </c>
-      <c r="C48" t="s" s="27">
+      <c r="C48" s="27" t="s">
         <v>235</v>
       </c>
-      <c r="D48" t="s" s="19">
+      <c r="D48" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="E48" t="s" s="19">
+      <c r="E48" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="F48" t="s" s="20">
+      <c r="F48" s="20" t="s">
         <v>243</v>
       </c>
       <c r="G48" s="28"/>
-    </row>
-    <row r="49" ht="144" customHeight="1">
-      <c r="A49" t="s" s="27">
+      <c r="H48" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="27" t="s">
         <v>244</v>
       </c>
-      <c r="B49" t="s" s="27">
+      <c r="B49" s="27" t="s">
         <v>245</v>
       </c>
-      <c r="C49" t="s" s="27">
+      <c r="C49" s="27" t="s">
         <v>246</v>
       </c>
-      <c r="D49" t="s" s="19">
+      <c r="D49" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="E49" t="s" s="19">
+      <c r="E49" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="F49" t="s" s="20">
+      <c r="F49" s="20" t="s">
         <v>249</v>
       </c>
       <c r="G49" s="28"/>
-    </row>
-    <row r="50" ht="144" customHeight="1">
-      <c r="A50" t="s" s="27">
+      <c r="H49" s="1">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="B50" t="s" s="27">
+      <c r="B50" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="C50" t="s" s="27">
+      <c r="C50" s="27" t="s">
         <v>246</v>
       </c>
-      <c r="D50" t="s" s="19">
+      <c r="D50" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="E50" t="s" s="19">
+      <c r="E50" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="F50" t="s" s="20">
+      <c r="F50" s="20" t="s">
         <v>254</v>
       </c>
       <c r="G50" s="28"/>
-    </row>
-    <row r="51" ht="160" customHeight="1">
-      <c r="A51" t="s" s="27">
+      <c r="H50" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="B51" t="s" s="27">
+      <c r="B51" s="27" t="s">
         <v>256</v>
       </c>
-      <c r="C51" t="s" s="27">
+      <c r="C51" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="D51" t="s" s="19">
+      <c r="D51" s="19" t="s">
         <v>258</v>
       </c>
-      <c r="E51" t="s" s="19">
+      <c r="E51" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="F51" t="s" s="20">
+      <c r="F51" s="20" t="s">
         <v>260</v>
       </c>
       <c r="G51" s="28"/>
-    </row>
-    <row r="52" ht="160" customHeight="1">
-      <c r="A52" t="s" s="27">
+      <c r="H51" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="B52" t="s" s="27">
+      <c r="B52" s="27" t="s">
         <v>262</v>
       </c>
-      <c r="C52" t="s" s="27">
+      <c r="C52" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="D52" t="s" s="19">
+      <c r="D52" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="E52" t="s" s="19">
+      <c r="E52" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="F52" t="s" s="20">
+      <c r="F52" s="20" t="s">
         <v>265</v>
       </c>
       <c r="G52" s="28"/>
-    </row>
-    <row r="53" ht="160" customHeight="1">
-      <c r="A53" t="s" s="27">
+      <c r="H52" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="B53" t="s" s="27">
+      <c r="B53" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="C53" t="s" s="27">
+      <c r="C53" s="27" t="s">
         <v>268</v>
       </c>
-      <c r="D53" t="s" s="19">
+      <c r="D53" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="E53" t="s" s="19">
+      <c r="E53" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="F53" t="s" s="20">
+      <c r="F53" s="20" t="s">
         <v>271</v>
       </c>
       <c r="G53" s="28"/>
-    </row>
-    <row r="54" ht="160" customHeight="1">
-      <c r="A54" t="s" s="27">
+      <c r="H53" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="160" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="27" t="s">
         <v>272</v>
       </c>
-      <c r="B54" t="s" s="27">
+      <c r="B54" s="27" t="s">
         <v>273</v>
       </c>
-      <c r="C54" t="s" s="27">
+      <c r="C54" s="27" t="s">
         <v>268</v>
       </c>
-      <c r="D54" t="s" s="19">
+      <c r="D54" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="E54" t="s" s="19">
+      <c r="E54" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="F54" t="s" s="20">
+      <c r="F54" s="20" t="s">
         <v>276</v>
       </c>
       <c r="G54" s="28"/>
-    </row>
-    <row r="55" ht="144" customHeight="1">
-      <c r="A55" t="s" s="27">
+      <c r="H54" s="1">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="27" t="s">
         <v>277</v>
       </c>
-      <c r="B55" t="s" s="27">
+      <c r="B55" s="27" t="s">
         <v>278</v>
       </c>
-      <c r="C55" t="s" s="27">
+      <c r="C55" s="27" t="s">
         <v>279</v>
       </c>
-      <c r="D55" t="s" s="19">
+      <c r="D55" s="19" t="s">
         <v>280</v>
       </c>
-      <c r="E55" t="s" s="19">
+      <c r="E55" s="19" t="s">
         <v>281</v>
       </c>
-      <c r="F55" t="s" s="20">
+      <c r="F55" s="20" t="s">
         <v>282</v>
       </c>
       <c r="G55" s="28"/>
-    </row>
-    <row r="56" ht="144" customHeight="1">
-      <c r="A56" t="s" s="27">
+      <c r="H55" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="144" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="27" t="s">
         <v>283</v>
       </c>
-      <c r="B56" t="s" s="27">
+      <c r="B56" s="27" t="s">
         <v>284</v>
       </c>
-      <c r="C56" t="s" s="27">
+      <c r="C56" s="27" t="s">
         <v>279</v>
       </c>
-      <c r="D56" t="s" s="19">
+      <c r="D56" s="19" t="s">
         <v>285</v>
       </c>
-      <c r="E56" t="s" s="19">
+      <c r="E56" s="19" t="s">
         <v>286</v>
       </c>
-      <c r="F56" t="s" s="20">
+      <c r="F56" s="20" t="s">
         <v>287</v>
       </c>
       <c r="G56" s="28"/>
+      <c r="H56" s="1">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>